<commit_message>
Update glossary spreadsheet and add short DE test dataset
</commit_message>
<xml_diff>
--- a/dataset/00_Glossary_Rotpunkt.xlsx
+++ b/dataset/00_Glossary_Rotpunkt.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Rotpunküchen\dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3844B938-C38C-4DC6-AC70-465186B999FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23BE7211-740F-4F48-8C74-05051355B438}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Glossary" sheetId="1" r:id="rId1"/>
@@ -905,7 +905,7 @@
     <col min="6" max="6" width="22" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="9" max="9" width="29.85546875" customWidth="1"/>
     <col min="10" max="10" width="14.140625" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>